<commit_message>
started a masonry walls and some minor excel stuff
</commit_message>
<xml_diff>
--- a/Masonry Code/Masonry_Tables.xlsx
+++ b/Masonry Code/Masonry_Tables.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8b45b1c4bb17244/ARCE/Masonry Code/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alisaleh/Desktop/Senior Collaborative Project/Senior-Project-Code/Masonry Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="62" documentId="8_{D9EF1D44-BA81-4FD3-BA4E-E5C19EFA8111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84736A22-3D78-4799-87BD-8F4B22CDA15B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94BBE933-9AF9-F64D-9BF8-3D87A9EB8F1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{42E9945D-B200-40E3-932A-4885E6232AB3}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="23260" windowHeight="12460" activeTab="3" xr2:uid="{42E9945D-B200-40E3-932A-4885E6232AB3}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebar_Size" sheetId="1" r:id="rId1"/>
     <sheet name="fr_beam" sheetId="2" r:id="rId2"/>
+    <sheet name="net_area_comp_strength_clay" sheetId="4" r:id="rId3"/>
+    <sheet name="net_area_comp_strength_concrete" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="12">
   <si>
     <t>Bar number</t>
   </si>
@@ -70,6 +72,9 @@
   </si>
   <si>
     <t>FGU</t>
+  </si>
+  <si>
+    <t>Comp Str</t>
   </si>
 </sst>
 </file>
@@ -122,10 +127,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -446,14 +447,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63BCD990-A294-466E-B602-A230ED151825}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" customWidth="1"/>
+    <col min="1" max="1" width="10.5" customWidth="1"/>
     <col min="2" max="2" width="11.33203125" customWidth="1"/>
-    <col min="3" max="3" width="9.88671875" customWidth="1"/>
+    <col min="3" max="3" width="9.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -464,7 +465,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>3</v>
       </c>
@@ -475,7 +476,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>4</v>
       </c>
@@ -486,7 +487,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>5</v>
       </c>
@@ -497,7 +498,7 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>6</v>
       </c>
@@ -508,7 +509,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>7</v>
       </c>
@@ -519,7 +520,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>8</v>
       </c>
@@ -530,7 +531,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>9</v>
       </c>
@@ -541,7 +542,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>10</v>
       </c>
@@ -552,7 +553,7 @@
         <v>1.27</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>11</v>
       </c>
@@ -571,12 +572,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DC4CD92-9491-4EE8-9665-AB292A9740BE}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.88671875" customWidth="1"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -590,7 +591,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -604,7 +605,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -618,7 +619,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -632,7 +633,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -644,6 +645,218 @@
       </c>
       <c r="D5">
         <v>200</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C19DDB4E-59DD-444F-A75A-CD09A8CAFA23}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1000</v>
+      </c>
+      <c r="B2">
+        <v>1700</v>
+      </c>
+      <c r="C2">
+        <v>1700</v>
+      </c>
+      <c r="D2">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1500</v>
+      </c>
+      <c r="B3">
+        <v>3350</v>
+      </c>
+      <c r="C3">
+        <v>3350</v>
+      </c>
+      <c r="D3">
+        <v>4150</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>2000</v>
+      </c>
+      <c r="B4">
+        <v>4950</v>
+      </c>
+      <c r="C4">
+        <v>4950</v>
+      </c>
+      <c r="D4">
+        <v>6200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>2500</v>
+      </c>
+      <c r="B5">
+        <v>6600</v>
+      </c>
+      <c r="C5">
+        <v>6600</v>
+      </c>
+      <c r="D5">
+        <v>8250</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>3000</v>
+      </c>
+      <c r="B6">
+        <v>8250</v>
+      </c>
+      <c r="C6">
+        <v>8250</v>
+      </c>
+      <c r="D6">
+        <v>10300</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>3500</v>
+      </c>
+      <c r="B7">
+        <v>9900</v>
+      </c>
+      <c r="C7">
+        <v>9900</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>4000</v>
+      </c>
+      <c r="B8">
+        <v>11500</v>
+      </c>
+      <c r="C8">
+        <v>11500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FD962C5-A8B9-DD4B-A585-8BE9192601DC}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1750</v>
+      </c>
+      <c r="D2">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2000</v>
+      </c>
+      <c r="B3">
+        <v>2000</v>
+      </c>
+      <c r="C3">
+        <v>2000</v>
+      </c>
+      <c r="D3">
+        <v>2650</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>2250</v>
+      </c>
+      <c r="B4">
+        <v>2600</v>
+      </c>
+      <c r="C4">
+        <v>2600</v>
+      </c>
+      <c r="D4">
+        <v>3400</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>2500</v>
+      </c>
+      <c r="B5">
+        <v>3250</v>
+      </c>
+      <c r="C5">
+        <v>3250</v>
+      </c>
+      <c r="D5">
+        <v>4350</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>2750</v>
+      </c>
+      <c r="B6">
+        <v>3900</v>
+      </c>
+      <c r="C6">
+        <v>3900</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>3000</v>
+      </c>
+      <c r="B7">
+        <v>4500</v>
+      </c>
+      <c r="C7">
+        <v>4500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
More work done on pm itneraction
</commit_message>
<xml_diff>
--- a/Masonry Code/Masonry_Tables.xlsx
+++ b/Masonry Code/Masonry_Tables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alisaleh/Desktop/Senior Collaborative Project/Senior-Project-Code/Masonry Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94BBE933-9AF9-F64D-9BF8-3D87A9EB8F1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91A26178-2D01-7046-A38E-5290F5339A34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="23260" windowHeight="12460" activeTab="3" xr2:uid="{42E9945D-B200-40E3-932A-4885E6232AB3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="11">
   <si>
     <t>Bar number</t>
   </si>
@@ -48,9 +48,6 @@
   </si>
   <si>
     <t>Area (in^2)</t>
-  </si>
-  <si>
-    <t>Description</t>
   </si>
   <si>
     <t>M</t>
@@ -578,22 +575,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="B1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>5</v>
-      </c>
-      <c r="D1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B2">
         <v>267</v>
@@ -607,7 +601,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>167</v>
@@ -621,7 +615,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4">
         <v>167</v>
@@ -635,7 +629,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5">
         <v>267</v>
@@ -659,16 +653,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>5</v>
-      </c>
-      <c r="D1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -775,16 +769,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>5</v>
-      </c>
-      <c r="D1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>